<commit_message>
Update renv and run spreadsheet
</commit_message>
<xml_diff>
--- a/data/turc_2026.xlsx
+++ b/data/turc_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/andy_wilson8_nhs_net/Documents/Git2/turc_run_2026/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B13B60BA-BA47-4A97-B586-A9431636BFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{B13B60BA-BA47-4A97-B586-A9431636BFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D875EC5-7511-43BE-BEDD-0DE2F02F485D}"/>
   <bookViews>
-    <workbookView xWindow="28980" yWindow="-7020" windowWidth="29040" windowHeight="15720" xr2:uid="{AF5544F7-E203-44AA-819B-E456A0906A7C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{AF5544F7-E203-44AA-819B-E456A0906A7C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -433,7 +433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DEE0951-953A-4811-8EB6-CF908CA14FD1}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" bestFit="1" customWidth="1"/>
@@ -489,6 +489,32 @@
       </c>
       <c r="H2">
         <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="1">
+        <v>46035</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Align renv repo and data updates
</commit_message>
<xml_diff>
--- a/data/turc_2026.xlsx
+++ b/data/turc_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/andy_wilson8_nhs_net/Documents/Git2/turc_run_2026/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{B13B60BA-BA47-4A97-B586-A9431636BFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D875EC5-7511-43BE-BEDD-0DE2F02F485D}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{B13B60BA-BA47-4A97-B586-A9431636BFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8BEA507-B90F-428D-BE41-AC650A3CA5D8}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{AF5544F7-E203-44AA-819B-E456A0906A7C}"/>
   </bookViews>
@@ -496,7 +496,7 @@
         <v>46035</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>5.9</v>
       </c>
       <c r="C3">
         <v>1</v>

</xml_diff>

<commit_message>
Fix distance in spreadsheet
</commit_message>
<xml_diff>
--- a/data/turc_2026.xlsx
+++ b/data/turc_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/andy_wilson8_nhs_net/Documents/Git2/turc_run_2026/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{B13B60BA-BA47-4A97-B586-A9431636BFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8BEA507-B90F-428D-BE41-AC650A3CA5D8}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{B13B60BA-BA47-4A97-B586-A9431636BFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3710BF84-6F80-4BF9-818D-D37138FD13C8}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{AF5544F7-E203-44AA-819B-E456A0906A7C}"/>
   </bookViews>
@@ -496,7 +496,7 @@
         <v>46035</v>
       </c>
       <c r="B3">
-        <v>5.9</v>
+        <v>5</v>
       </c>
       <c r="C3">
         <v>1</v>

</xml_diff>

<commit_message>
Updated dataset with latest run
</commit_message>
<xml_diff>
--- a/data/turc_2026.xlsx
+++ b/data/turc_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/andy_wilson8_nhs_net/Documents/Git2/turc_run_2026/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{B13B60BA-BA47-4A97-B586-A9431636BFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7DB7B22-77EA-462E-A587-A005EE8046D9}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="8_{B13B60BA-BA47-4A97-B586-A9431636BFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F65483A9-FE77-4903-89D4-D67551813221}"/>
   <bookViews>
-    <workbookView xWindow="180" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{AF5544F7-E203-44AA-819B-E456A0906A7C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{AF5544F7-E203-44AA-819B-E456A0906A7C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -433,7 +433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DEE0951-953A-4811-8EB6-CF908CA14FD1}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" bestFit="1" customWidth="1"/>
@@ -566,6 +566,32 @@
         <v>0</v>
       </c>
       <c r="H5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" s="1">
+        <v>46071</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
         <v>0</v>
       </c>
     </row>

</xml_diff>